<commit_message>
Patch IDOR (Enkripsi ID) untuk modul SuratPermohonan, PekerjaanSda, dan Master Data
</commit_message>
<xml_diff>
--- a/public/usulan.xlsx
+++ b/public/usulan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\program file\Project Kantor\App-Reses\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F1C19A2-5EE4-4C3D-AB7B-FDB67A907098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44FE238-16F0-4C9C-A1D0-F581AC8907B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{45687CCE-BB77-4D6D-838D-A18CBCE99500}"/>
   </bookViews>
@@ -2291,7 +2291,7 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2313,6 +2313,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF6F8F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2434,7 +2446,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2548,6 +2560,18 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3015,7 +3039,7 @@
       <c r="B4" s="18">
         <v>46028</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="39" t="s">
         <v>26</v>
       </c>
       <c r="D4" s="20" t="s">
@@ -3048,7 +3072,7 @@
       <c r="B5" s="12">
         <v>46041</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="39" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="14" t="s">
@@ -3081,7 +3105,7 @@
       <c r="B6" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="39" t="s">
         <v>35</v>
       </c>
       <c r="D6" s="20" t="s">
@@ -3114,7 +3138,7 @@
       <c r="B7" s="12">
         <v>46041</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="39" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="14" t="s">
@@ -3149,7 +3173,7 @@
       <c r="B8" s="18">
         <v>46042</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="39" t="s">
         <v>47</v>
       </c>
       <c r="D8" s="20" t="s">
@@ -3182,7 +3206,7 @@
       <c r="B9" s="12">
         <v>46037</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="39" t="s">
         <v>52</v>
       </c>
       <c r="D9" s="14" t="s">
@@ -3215,7 +3239,7 @@
       <c r="B10" s="18">
         <v>46042</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="39" t="s">
         <v>59</v>
       </c>
       <c r="D10" s="20" t="s">
@@ -3248,7 +3272,7 @@
       <c r="B11" s="12">
         <v>46045</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="39" t="s">
         <v>65</v>
       </c>
       <c r="D11" s="14" t="s">
@@ -3281,7 +3305,7 @@
       <c r="B12" s="18">
         <v>46042</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="39" t="s">
         <v>69</v>
       </c>
       <c r="D12" s="20" t="s">
@@ -3314,7 +3338,7 @@
       <c r="B13" s="12">
         <v>46040</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="39" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="14" t="s">
@@ -3347,7 +3371,7 @@
       <c r="B14" s="18">
         <v>46044</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="40" t="s">
         <v>77</v>
       </c>
       <c r="D14" s="20" t="s">
@@ -3380,7 +3404,7 @@
       <c r="B15" s="12">
         <v>46044</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="40" t="s">
         <v>77</v>
       </c>
       <c r="D15" s="14" t="s">
@@ -3415,7 +3439,7 @@
       <c r="B16" s="18">
         <v>46030</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="39" t="s">
         <v>82</v>
       </c>
       <c r="D16" s="20" t="s">
@@ -3448,7 +3472,7 @@
       <c r="B17" s="12">
         <v>46042</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="39" t="s">
         <v>86</v>
       </c>
       <c r="D17" s="14" t="s">
@@ -3481,7 +3505,7 @@
       <c r="B18" s="18">
         <v>46043</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="39" t="s">
         <v>91</v>
       </c>
       <c r="D18" s="20" t="s">
@@ -3514,7 +3538,7 @@
       <c r="B19" s="12">
         <v>46048</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="39" t="s">
         <v>94</v>
       </c>
       <c r="D19" s="14" t="s">
@@ -3547,7 +3571,7 @@
       <c r="B20" s="18">
         <v>46049</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="39" t="s">
         <v>98</v>
       </c>
       <c r="D20" s="20" t="s">
@@ -3580,7 +3604,7 @@
       <c r="B21" s="12">
         <v>46049</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="39" t="s">
         <v>103</v>
       </c>
       <c r="D21" s="14" t="s">
@@ -3613,7 +3637,7 @@
       <c r="B22" s="18">
         <v>45894</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="40" t="s">
         <v>106</v>
       </c>
       <c r="D22" s="20" t="s">
@@ -3646,7 +3670,7 @@
       <c r="B23" s="12">
         <v>45686</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="39" t="s">
         <v>110</v>
       </c>
       <c r="D23" s="14" t="s">
@@ -3672,14 +3696,14 @@
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
     </row>
-    <row r="24" spans="1:13" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="17">
         <v>127</v>
       </c>
       <c r="B24" s="18">
         <v>46051</v>
       </c>
-      <c r="C24" s="19" t="s">
+      <c r="C24" s="39" t="s">
         <v>114</v>
       </c>
       <c r="D24" s="20" t="s">
@@ -3712,7 +3736,7 @@
       <c r="B25" s="12">
         <v>45895</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="39" t="s">
         <v>120</v>
       </c>
       <c r="D25" s="14" t="s">
@@ -3745,7 +3769,7 @@
       <c r="B26" s="18">
         <v>46051</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="39" t="s">
         <v>125</v>
       </c>
       <c r="D26" s="20" t="s">
@@ -3778,7 +3802,7 @@
       <c r="B27" s="12">
         <v>46056</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="39" t="s">
         <v>129</v>
       </c>
       <c r="D27" s="14" t="s">
@@ -3811,7 +3835,7 @@
       <c r="B28" s="18">
         <v>46057</v>
       </c>
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="39" t="s">
         <v>133</v>
       </c>
       <c r="D28" s="20" t="s">
@@ -3844,7 +3868,7 @@
       <c r="B29" s="12">
         <v>46057</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="39" t="s">
         <v>137</v>
       </c>
       <c r="D29" s="14" t="s">
@@ -3877,7 +3901,7 @@
       <c r="B30" s="18">
         <v>46059</v>
       </c>
-      <c r="C30" s="19" t="s">
+      <c r="C30" s="39" t="s">
         <v>141</v>
       </c>
       <c r="D30" s="20" t="s">
@@ -3910,7 +3934,7 @@
       <c r="B31" s="12">
         <v>46049</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="39" t="s">
         <v>145</v>
       </c>
       <c r="D31" s="14" t="s">
@@ -3943,7 +3967,7 @@
       <c r="B32" s="18">
         <v>46052</v>
       </c>
-      <c r="C32" s="19" t="s">
+      <c r="C32" s="39" t="s">
         <v>149</v>
       </c>
       <c r="D32" s="20" t="s">
@@ -3976,7 +4000,7 @@
       <c r="B33" s="12">
         <v>46058</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="39" t="s">
         <v>154</v>
       </c>
       <c r="D33" s="14" t="s">
@@ -4102,7 +4126,7 @@
       <c r="B37" s="12">
         <v>46058</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="39" t="s">
         <v>169</v>
       </c>
       <c r="D37" s="14" t="s">
@@ -4135,13 +4159,13 @@
       <c r="B38" s="18">
         <v>46055</v>
       </c>
-      <c r="C38" s="19" t="s">
+      <c r="C38" s="39" t="s">
         <v>172</v>
       </c>
       <c r="D38" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="E38" s="31" t="s">
+      <c r="E38" s="41" t="s">
         <v>15</v>
       </c>
       <c r="F38" s="20" t="s">
@@ -4168,7 +4192,7 @@
       <c r="B39" s="12">
         <v>46064</v>
       </c>
-      <c r="C39" s="13" t="s">
+      <c r="C39" s="39" t="s">
         <v>176</v>
       </c>
       <c r="D39" s="14" t="s">
@@ -4201,7 +4225,7 @@
       <c r="B40" s="18">
         <v>46066</v>
       </c>
-      <c r="C40" s="19" t="s">
+      <c r="C40" s="39" t="s">
         <v>179</v>
       </c>
       <c r="D40" s="20" t="s">
@@ -4234,7 +4258,7 @@
       <c r="B41" s="12">
         <v>46064</v>
       </c>
-      <c r="C41" s="13" t="s">
+      <c r="C41" s="39" t="s">
         <v>183</v>
       </c>
       <c r="D41" s="14" t="s">
@@ -4267,7 +4291,7 @@
       <c r="B42" s="18">
         <v>46064</v>
       </c>
-      <c r="C42" s="19" t="s">
+      <c r="C42" s="39" t="s">
         <v>186</v>
       </c>
       <c r="D42" s="20" t="s">
@@ -4300,7 +4324,7 @@
       <c r="B43" s="12">
         <v>46071</v>
       </c>
-      <c r="C43" s="13" t="s">
+      <c r="C43" s="39" t="s">
         <v>189</v>
       </c>
       <c r="D43" s="14" t="s">
@@ -4333,7 +4357,7 @@
       <c r="B44" s="18">
         <v>46063</v>
       </c>
-      <c r="C44" s="19" t="s">
+      <c r="C44" s="39" t="s">
         <v>192</v>
       </c>
       <c r="D44" s="20" t="s">
@@ -4366,7 +4390,7 @@
       <c r="B45" s="12">
         <v>46063</v>
       </c>
-      <c r="C45" s="13" t="s">
+      <c r="C45" s="39" t="s">
         <v>196</v>
       </c>
       <c r="D45" s="14" t="s">
@@ -4399,7 +4423,7 @@
       <c r="B46" s="18">
         <v>46073</v>
       </c>
-      <c r="C46" s="19" t="s">
+      <c r="C46" s="39" t="s">
         <v>199</v>
       </c>
       <c r="D46" s="20" t="s">
@@ -4432,7 +4456,7 @@
       <c r="B47" s="12">
         <v>46070</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="C47" s="39" t="s">
         <v>203</v>
       </c>
       <c r="D47" s="14" t="s">
@@ -4465,7 +4489,7 @@
       <c r="B48" s="18">
         <v>46063</v>
       </c>
-      <c r="C48" s="19" t="s">
+      <c r="C48" s="39" t="s">
         <v>207</v>
       </c>
       <c r="D48" s="20" t="s">
@@ -4500,7 +4524,7 @@
       <c r="B49" s="12">
         <v>46082</v>
       </c>
-      <c r="C49" s="13" t="s">
+      <c r="C49" s="39" t="s">
         <v>212</v>
       </c>
       <c r="D49" s="14" t="s">
@@ -4533,7 +4557,7 @@
       <c r="B50" s="18">
         <v>46083</v>
       </c>
-      <c r="C50" s="19" t="s">
+      <c r="C50" s="39" t="s">
         <v>216</v>
       </c>
       <c r="D50" s="20" t="s">
@@ -4566,7 +4590,7 @@
       <c r="B51" s="12">
         <v>46084</v>
       </c>
-      <c r="C51" s="13" t="s">
+      <c r="C51" s="39" t="s">
         <v>219</v>
       </c>
       <c r="D51" s="14" t="s">
@@ -4599,7 +4623,7 @@
       <c r="B52" s="18">
         <v>46078</v>
       </c>
-      <c r="C52" s="19" t="s">
+      <c r="C52" s="39" t="s">
         <v>223</v>
       </c>
       <c r="D52" s="20" t="s">
@@ -4632,7 +4656,7 @@
       <c r="B53" s="12">
         <v>46076</v>
       </c>
-      <c r="C53" s="13" t="s">
+      <c r="C53" s="40" t="s">
         <v>226</v>
       </c>
       <c r="D53" s="14" t="s">
@@ -4667,7 +4691,7 @@
       <c r="B54" s="18">
         <v>46073</v>
       </c>
-      <c r="C54" s="19" t="s">
+      <c r="C54" s="39" t="s">
         <v>231</v>
       </c>
       <c r="D54" s="20" t="s">
@@ -4700,7 +4724,7 @@
       <c r="B55" s="12">
         <v>46077</v>
       </c>
-      <c r="C55" s="13" t="s">
+      <c r="C55" s="39" t="s">
         <v>235</v>
       </c>
       <c r="D55" s="14" t="s">
@@ -4733,7 +4757,7 @@
       <c r="B56" s="18">
         <v>46064</v>
       </c>
-      <c r="C56" s="19" t="s">
+      <c r="C56" s="39" t="s">
         <v>237</v>
       </c>
       <c r="D56" s="20" t="s">
@@ -4766,7 +4790,7 @@
       <c r="B57" s="12">
         <v>46078</v>
       </c>
-      <c r="C57" s="13" t="s">
+      <c r="C57" s="39" t="s">
         <v>240</v>
       </c>
       <c r="D57" s="14" t="s">
@@ -4799,7 +4823,7 @@
       <c r="B58" s="18">
         <v>46078</v>
       </c>
-      <c r="C58" s="19" t="s">
+      <c r="C58" s="39" t="s">
         <v>243</v>
       </c>
       <c r="D58" s="20" t="s">
@@ -4832,7 +4856,7 @@
       <c r="B59" s="12">
         <v>46086</v>
       </c>
-      <c r="C59" s="13" t="s">
+      <c r="C59" s="39" t="s">
         <v>247</v>
       </c>
       <c r="D59" s="14" t="s">
@@ -4865,7 +4889,7 @@
       <c r="B60" s="18">
         <v>46091</v>
       </c>
-      <c r="C60" s="19" t="s">
+      <c r="C60" s="39" t="s">
         <v>251</v>
       </c>
       <c r="D60" s="20" t="s">
@@ -4891,14 +4915,14 @@
       <c r="L60" s="22"/>
       <c r="M60" s="22"/>
     </row>
-    <row r="61" spans="1:13" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
         <v>164</v>
       </c>
       <c r="B61" s="12">
         <v>46092</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="C61" s="39" t="s">
         <v>254</v>
       </c>
       <c r="D61" s="14" t="s">
@@ -4931,7 +4955,7 @@
       <c r="B62" s="18">
         <v>46084</v>
       </c>
-      <c r="C62" s="19" t="s">
+      <c r="C62" s="39" t="s">
         <v>219</v>
       </c>
       <c r="D62" s="20" t="s">
@@ -4964,7 +4988,7 @@
       <c r="B63" s="12">
         <v>46090</v>
       </c>
-      <c r="C63" s="13" t="s">
+      <c r="C63" s="39" t="s">
         <v>260</v>
       </c>
       <c r="D63" s="14" t="s">
@@ -4997,7 +5021,7 @@
       <c r="B64" s="18">
         <v>46090</v>
       </c>
-      <c r="C64" s="19" t="s">
+      <c r="C64" s="39" t="s">
         <v>263</v>
       </c>
       <c r="D64" s="20" t="s">
@@ -5063,7 +5087,7 @@
       <c r="B66" s="18">
         <v>46086</v>
       </c>
-      <c r="C66" s="19" t="s">
+      <c r="C66" s="39" t="s">
         <v>271</v>
       </c>
       <c r="D66" s="20" t="s">
@@ -5096,7 +5120,7 @@
       <c r="B67" s="12">
         <v>46093</v>
       </c>
-      <c r="C67" s="13" t="s">
+      <c r="C67" s="39" t="s">
         <v>275</v>
       </c>
       <c r="D67" s="14" t="s">
@@ -5129,7 +5153,7 @@
       <c r="B68" s="18">
         <v>46112</v>
       </c>
-      <c r="C68" s="19" t="s">
+      <c r="C68" s="39" t="s">
         <v>278</v>
       </c>
       <c r="D68" s="20" t="s">
@@ -5155,14 +5179,14 @@
       <c r="L68" s="22"/>
       <c r="M68" s="22"/>
     </row>
-    <row r="69" spans="1:13" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:13" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="11">
         <v>172</v>
       </c>
       <c r="B69" s="12">
         <v>46115</v>
       </c>
-      <c r="C69" s="13" t="s">
+      <c r="C69" s="39" t="s">
         <v>282</v>
       </c>
       <c r="D69" s="14" t="s">
@@ -5195,7 +5219,7 @@
       <c r="B70" s="18">
         <v>46118</v>
       </c>
-      <c r="C70" s="19" t="s">
+      <c r="C70" s="39" t="s">
         <v>286</v>
       </c>
       <c r="D70" s="20" t="s">
@@ -5228,7 +5252,7 @@
       <c r="B71" s="12">
         <v>46113</v>
       </c>
-      <c r="C71" s="13" t="s">
+      <c r="C71" s="39" t="s">
         <v>290</v>
       </c>
       <c r="D71" s="14" t="s">
@@ -5261,7 +5285,7 @@
       <c r="B72" s="18">
         <v>46119</v>
       </c>
-      <c r="C72" s="19" t="s">
+      <c r="C72" s="39" t="s">
         <v>293</v>
       </c>
       <c r="D72" s="20" t="s">
@@ -5294,7 +5318,7 @@
       <c r="B73" s="12">
         <v>46113</v>
       </c>
-      <c r="C73" s="13" t="s">
+      <c r="C73" s="39" t="s">
         <v>297</v>
       </c>
       <c r="D73" s="14" t="s">
@@ -5327,7 +5351,7 @@
       <c r="B74" s="18">
         <v>46123</v>
       </c>
-      <c r="C74" s="19" t="s">
+      <c r="C74" s="39" t="s">
         <v>300</v>
       </c>
       <c r="D74" s="20" t="s">
@@ -5360,7 +5384,7 @@
       <c r="B75" s="12">
         <v>46073</v>
       </c>
-      <c r="C75" s="13" t="s">
+      <c r="C75" s="39" t="s">
         <v>302</v>
       </c>
       <c r="D75" s="14" t="s">
@@ -5393,7 +5417,7 @@
       <c r="B76" s="18">
         <v>46036</v>
       </c>
-      <c r="C76" s="19" t="s">
+      <c r="C76" s="39" t="s">
         <v>305</v>
       </c>
       <c r="D76" s="20" t="s">
@@ -5426,7 +5450,7 @@
       <c r="B77" s="12">
         <v>46043</v>
       </c>
-      <c r="C77" s="13" t="s">
+      <c r="C77" s="39" t="s">
         <v>309</v>
       </c>
       <c r="D77" s="14" t="s">
@@ -5459,13 +5483,13 @@
       <c r="B78" s="18">
         <v>46121</v>
       </c>
-      <c r="C78" s="19" t="s">
+      <c r="C78" s="39" t="s">
         <v>312</v>
       </c>
       <c r="D78" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="E78" s="29" t="s">
+      <c r="E78" s="42" t="s">
         <v>54</v>
       </c>
       <c r="F78" s="20" t="s">
@@ -5492,7 +5516,7 @@
       <c r="B79" s="12">
         <v>46111</v>
       </c>
-      <c r="C79" s="13" t="s">
+      <c r="C79" s="39" t="s">
         <v>316</v>
       </c>
       <c r="D79" s="14" t="s">
@@ -5525,7 +5549,7 @@
       <c r="B80" s="18">
         <v>46122</v>
       </c>
-      <c r="C80" s="19" t="s">
+      <c r="C80" s="39" t="s">
         <v>320</v>
       </c>
       <c r="D80" s="20" t="s">
@@ -5558,7 +5582,7 @@
       <c r="B81" s="12">
         <v>46126</v>
       </c>
-      <c r="C81" s="13" t="s">
+      <c r="C81" s="39" t="s">
         <v>323</v>
       </c>
       <c r="D81" s="14" t="s">
@@ -5624,7 +5648,7 @@
       <c r="B83" s="12">
         <v>46046</v>
       </c>
-      <c r="C83" s="13" t="s">
+      <c r="C83" s="39" t="s">
         <v>329</v>
       </c>
       <c r="D83" s="14" t="s">
@@ -5657,7 +5681,7 @@
       <c r="B84" s="18">
         <v>46125</v>
       </c>
-      <c r="C84" s="19" t="s">
+      <c r="C84" s="39" t="s">
         <v>333</v>
       </c>
       <c r="D84" s="20" t="s">
@@ -5690,7 +5714,7 @@
       <c r="B85" s="12">
         <v>46127</v>
       </c>
-      <c r="C85" s="13" t="s">
+      <c r="C85" s="39" t="s">
         <v>337</v>
       </c>
       <c r="D85" s="14" t="s">
@@ -5723,7 +5747,7 @@
       <c r="B86" s="18">
         <v>46126</v>
       </c>
-      <c r="C86" s="19" t="s">
+      <c r="C86" s="39" t="s">
         <v>340</v>
       </c>
       <c r="D86" s="20" t="s">
@@ -5756,7 +5780,7 @@
       <c r="B87" s="12">
         <v>46122</v>
       </c>
-      <c r="C87" s="13" t="s">
+      <c r="C87" s="39" t="s">
         <v>342</v>
       </c>
       <c r="D87" s="14" t="s">
@@ -5789,7 +5813,7 @@
       <c r="B88" s="18">
         <v>46128</v>
       </c>
-      <c r="C88" s="19" t="s">
+      <c r="C88" s="39" t="s">
         <v>345</v>
       </c>
       <c r="D88" s="20" t="s">
@@ -5822,7 +5846,7 @@
       <c r="B89" s="12">
         <v>46125</v>
       </c>
-      <c r="C89" s="13" t="s">
+      <c r="C89" s="39" t="s">
         <v>347</v>
       </c>
       <c r="D89" s="14" t="s">
@@ -5855,7 +5879,7 @@
       <c r="B90" s="18">
         <v>46128</v>
       </c>
-      <c r="C90" s="19" t="s">
+      <c r="C90" s="39" t="s">
         <v>350</v>
       </c>
       <c r="D90" s="20" t="s">
@@ -5888,7 +5912,7 @@
       <c r="B91" s="12">
         <v>46134</v>
       </c>
-      <c r="C91" s="13" t="s">
+      <c r="C91" s="39" t="s">
         <v>354</v>
       </c>
       <c r="D91" s="14" t="s">
@@ -5921,7 +5945,7 @@
       <c r="B92" s="18">
         <v>46135</v>
       </c>
-      <c r="C92" s="19" t="s">
+      <c r="C92" s="39" t="s">
         <v>358</v>
       </c>
       <c r="D92" s="20" t="s">
@@ -5954,7 +5978,7 @@
       <c r="B93" s="12">
         <v>46136</v>
       </c>
-      <c r="C93" s="13" t="s">
+      <c r="C93" s="39" t="s">
         <v>362</v>
       </c>
       <c r="D93" s="14" t="s">
@@ -5987,7 +6011,7 @@
       <c r="B94" s="18">
         <v>46132</v>
       </c>
-      <c r="C94" s="19" t="s">
+      <c r="C94" s="39" t="s">
         <v>366</v>
       </c>
       <c r="D94" s="20" t="s">
@@ -6020,7 +6044,7 @@
       <c r="B95" s="12">
         <v>46142</v>
       </c>
-      <c r="C95" s="13" t="s">
+      <c r="C95" s="39" t="s">
         <v>369</v>
       </c>
       <c r="D95" s="14" t="s">
@@ -6053,7 +6077,7 @@
       <c r="B96" s="18">
         <v>46141</v>
       </c>
-      <c r="C96" s="19" t="s">
+      <c r="C96" s="39" t="s">
         <v>372</v>
       </c>
       <c r="D96" s="20" t="s">
@@ -6086,7 +6110,7 @@
       <c r="B97" s="12">
         <v>46132</v>
       </c>
-      <c r="C97" s="13" t="s">
+      <c r="C97" s="39" t="s">
         <v>375</v>
       </c>
       <c r="D97" s="14" t="s">
@@ -6119,13 +6143,13 @@
       <c r="B98" s="18">
         <v>46106</v>
       </c>
-      <c r="C98" s="19" t="s">
+      <c r="C98" s="39" t="s">
         <v>378</v>
       </c>
       <c r="D98" s="20" t="s">
         <v>379</v>
       </c>
-      <c r="E98" s="31" t="s">
+      <c r="E98" s="41" t="s">
         <v>15</v>
       </c>
       <c r="F98" s="20" t="s">
@@ -6185,7 +6209,7 @@
       <c r="B100" s="18">
         <v>46141</v>
       </c>
-      <c r="C100" s="19" t="s">
+      <c r="C100" s="39" t="s">
         <v>385</v>
       </c>
       <c r="D100" s="20" t="s">
@@ -6220,7 +6244,7 @@
       <c r="B101" s="12">
         <v>46142</v>
       </c>
-      <c r="C101" s="13" t="s">
+      <c r="C101" s="39" t="s">
         <v>388</v>
       </c>
       <c r="D101" s="14" t="s">
@@ -6253,7 +6277,7 @@
       <c r="B102" s="18">
         <v>46146</v>
       </c>
-      <c r="C102" s="19" t="s">
+      <c r="C102" s="39" t="s">
         <v>391</v>
       </c>
       <c r="D102" s="20" t="s">
@@ -6286,7 +6310,7 @@
       <c r="B103" s="12">
         <v>46142</v>
       </c>
-      <c r="C103" s="13" t="s">
+      <c r="C103" s="39" t="s">
         <v>395</v>
       </c>
       <c r="D103" s="14" t="s">
@@ -6319,7 +6343,7 @@
       <c r="B104" s="18">
         <v>46142</v>
       </c>
-      <c r="C104" s="19" t="s">
+      <c r="C104" s="39" t="s">
         <v>399</v>
       </c>
       <c r="D104" s="20" t="s">
@@ -6352,7 +6376,7 @@
       <c r="B105" s="12">
         <v>46142</v>
       </c>
-      <c r="C105" s="13" t="s">
+      <c r="C105" s="39" t="s">
         <v>402</v>
       </c>
       <c r="D105" s="14" t="s">
@@ -6385,7 +6409,7 @@
       <c r="B106" s="18">
         <v>46148</v>
       </c>
-      <c r="C106" s="19" t="s">
+      <c r="C106" s="39" t="s">
         <v>405</v>
       </c>
       <c r="D106" s="20" t="s">
@@ -6418,7 +6442,7 @@
       <c r="B107" s="12">
         <v>46049</v>
       </c>
-      <c r="C107" s="13" t="s">
+      <c r="C107" s="39" t="s">
         <v>407</v>
       </c>
       <c r="D107" s="14" t="s">
@@ -6453,7 +6477,7 @@
       <c r="B108" s="18">
         <v>46049</v>
       </c>
-      <c r="C108" s="19" t="s">
+      <c r="C108" s="39" t="s">
         <v>411</v>
       </c>
       <c r="D108" s="20" t="s">
@@ -6488,7 +6512,7 @@
       <c r="B109" s="12">
         <v>46050</v>
       </c>
-      <c r="C109" s="13" t="s">
+      <c r="C109" s="39" t="s">
         <v>417</v>
       </c>
       <c r="D109" s="14" t="s">
@@ -6523,7 +6547,7 @@
       <c r="B110" s="18">
         <v>46063</v>
       </c>
-      <c r="C110" s="19" t="s">
+      <c r="C110" s="39" t="s">
         <v>207</v>
       </c>
       <c r="D110" s="20" t="s">
@@ -6698,7 +6722,7 @@
       <c r="B115" s="12">
         <v>46076</v>
       </c>
-      <c r="C115" s="13" t="s">
+      <c r="C115" s="40" t="s">
         <v>226</v>
       </c>
       <c r="D115" s="14" t="s">
@@ -6897,7 +6921,7 @@
       <c r="L120" s="22"/>
       <c r="M120" s="22"/>
     </row>
-    <row r="121" spans="1:13" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:13" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A121" s="11">
         <v>224</v>
       </c>
@@ -6930,7 +6954,7 @@
       <c r="L121" s="16"/>
       <c r="M121" s="16"/>
     </row>
-    <row r="122" spans="1:13" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:13" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A122" s="17">
         <v>225</v>
       </c>

</xml_diff>